<commit_message>
Rebuild index after corruption
</commit_message>
<xml_diff>
--- a/eth_purchases.xlsx
+++ b/eth_purchases.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,7 +464,7 @@
         <v>45851</v>
       </c>
       <c r="B2" t="n">
-        <v>163123</v>
+        <v>163142</v>
       </c>
       <c r="C2" t="n">
         <v>455776464</v>
@@ -473,7 +473,7 @@
         <v>2973.35888671875</v>
       </c>
       <c r="E2" t="n">
-        <v>13.22403266279382</v>
+        <v>13.22496228560634</v>
       </c>
     </row>
     <row r="3">
@@ -481,7 +481,7 @@
         <v>45858</v>
       </c>
       <c r="B3" t="n">
-        <v>137545</v>
+        <v>137515</v>
       </c>
       <c r="C3" t="n">
         <v>486978072</v>
@@ -490,7 +490,7 @@
         <v>3759.471435546875</v>
       </c>
       <c r="E3" t="n">
-        <v>12.14307611038233</v>
+        <v>12.14189821054058</v>
       </c>
     </row>
     <row r="4">
@@ -498,7 +498,7 @@
         <v>45865</v>
       </c>
       <c r="B4" t="n">
-        <v>266112</v>
+        <v>266119</v>
       </c>
       <c r="C4" t="n">
         <v>967982400</v>
@@ -507,7 +507,7 @@
         <v>3875.24658203125</v>
       </c>
       <c r="E4" t="n">
-        <v>16.8903458655477</v>
+        <v>16.89077172424776</v>
       </c>
     </row>
     <row r="5">
@@ -515,7 +515,7 @@
         <v>45872</v>
       </c>
       <c r="B5" t="n">
-        <v>58203</v>
+        <v>58208</v>
       </c>
       <c r="C5" t="n">
         <v>203244876</v>
@@ -524,7 +524,7 @@
         <v>3497.379150390625</v>
       </c>
       <c r="E5" t="n">
-        <v>7.899125219607736</v>
+        <v>7.899559777513748</v>
       </c>
     </row>
     <row r="6">
@@ -541,7 +541,7 @@
         <v>3683.920654296875</v>
       </c>
       <c r="E6" t="n">
-        <v>14.9380710547352</v>
+        <v>14.93825121853242</v>
       </c>
     </row>
     <row r="7">
@@ -558,7 +558,7 @@
         <v>4226.966796875</v>
       </c>
       <c r="E7" t="n">
-        <v>18.4382124370072</v>
+        <v>18.43843481500731</v>
       </c>
     </row>
     <row r="8">
@@ -566,7 +566,7 @@
         <v>45886</v>
       </c>
       <c r="B8" t="n">
-        <v>373119</v>
+        <v>373110</v>
       </c>
       <c r="C8" t="n">
         <v>1621595148</v>
@@ -592,7 +592,7 @@
         <v>4372.98779296875</v>
       </c>
       <c r="E9" t="n">
-        <v>14.29168508899322</v>
+        <v>14.29185745691441</v>
       </c>
     </row>
     <row r="10">
@@ -609,7 +609,7 @@
         <v>4507.177734375</v>
       </c>
       <c r="E10" t="n">
-        <v>9.190615970743885</v>
+        <v>9.190726816131217</v>
       </c>
     </row>
     <row r="11">
@@ -626,7 +626,7 @@
         <v>4325.36572265625</v>
       </c>
       <c r="E11" t="n">
-        <v>8.923884772639907</v>
+        <v>8.923992401058642</v>
       </c>
     </row>
     <row r="12">
@@ -643,7 +643,7 @@
         <v>4308.072265625</v>
       </c>
       <c r="E12" t="n">
-        <v>14.73280980151191</v>
+        <v>14.73298748971193</v>
       </c>
     </row>
     <row r="13">
@@ -651,7 +651,7 @@
         <v>45915</v>
       </c>
       <c r="B13" t="n">
-        <v>81682</v>
+        <v>82233</v>
       </c>
       <c r="C13" t="n">
         <v>369154256</v>
@@ -660,7 +660,7 @@
         <v>4526.8203125</v>
       </c>
       <c r="E13" t="n">
-        <v>9.357708118983352</v>
+        <v>9.389330327609359</v>
       </c>
     </row>
     <row r="14">
@@ -668,7 +668,7 @@
         <v>45922</v>
       </c>
       <c r="B14" t="n">
-        <v>264929</v>
+        <v>264378</v>
       </c>
       <c r="C14" t="n">
         <v>1181053482</v>
@@ -677,7 +677,7 @@
         <v>4202.87744140625</v>
       </c>
       <c r="E14" t="n">
-        <v>16.85276106040236</v>
+        <v>16.83542977611688</v>
       </c>
     </row>
     <row r="15">
@@ -694,7 +694,7 @@
         <v>4217.341796875</v>
       </c>
       <c r="E15" t="n">
-        <v>15.86711235595991</v>
+        <v>15.86730372465821</v>
       </c>
     </row>
     <row r="16">
@@ -711,7 +711,7 @@
         <v>4687.771484375</v>
       </c>
       <c r="E16" t="n">
-        <v>13.86235788517988</v>
+        <v>13.86252507510861</v>
       </c>
     </row>
     <row r="17">
@@ -728,7 +728,7 @@
         <v>4245.4677734375</v>
       </c>
       <c r="E17" t="n">
-        <v>14.71708400541464</v>
+        <v>14.71726150395034</v>
       </c>
     </row>
     <row r="18">
@@ -745,7 +745,7 @@
         <v>3980.76025390625</v>
       </c>
       <c r="E18" t="n">
-        <v>14.78209891758341</v>
+        <v>14.78227720024535</v>
       </c>
     </row>
     <row r="19">
@@ -762,7 +762,7 @@
         <v>4120.1220703125</v>
       </c>
       <c r="E19" t="n">
-        <v>9.08880374246251</v>
+        <v>9.088913359921712</v>
       </c>
     </row>
     <row r="20">
@@ -779,7 +779,7 @@
         <v>3602.30810546875</v>
       </c>
       <c r="E20" t="n">
-        <v>9.396065282374204</v>
+        <v>9.396178605626851</v>
       </c>
     </row>
     <row r="21">
@@ -787,16 +787,16 @@
         <v>45971</v>
       </c>
       <c r="B21" t="n">
-        <v>110301</v>
+        <v>110288</v>
       </c>
       <c r="C21" t="n">
-        <v>380538450</v>
+        <v>380489600</v>
       </c>
       <c r="D21" t="n">
         <v>3568.4599609375</v>
       </c>
       <c r="E21" t="n">
-        <v>10.87416799615108</v>
+        <v>10.87365830878528</v>
       </c>
     </row>
     <row r="22">
@@ -804,16 +804,16 @@
         <v>45978</v>
       </c>
       <c r="B22" t="n">
-        <v>54156</v>
+        <v>54176</v>
       </c>
       <c r="C22" t="n">
-        <v>171132960</v>
+        <v>171199960</v>
       </c>
       <c r="D22" t="n">
         <v>3024.538818359375</v>
       </c>
       <c r="E22" t="n">
-        <v>7.619554908713937</v>
+        <v>7.621053657199689</v>
       </c>
     </row>
     <row r="23">
@@ -830,7 +830,7 @@
         <v>2952.71337890625</v>
       </c>
       <c r="E23" t="n">
-        <v>8.651719998404761</v>
+        <v>8.651824344322094</v>
       </c>
     </row>
     <row r="24">
@@ -847,7 +847,7 @@
         <v>2800.18896484375</v>
       </c>
       <c r="E24" t="n">
-        <v>10.18684047888324</v>
+        <v>10.18696333944908</v>
       </c>
     </row>
     <row r="25">
@@ -864,7 +864,755 @@
         <v>3125.197998046875</v>
       </c>
       <c r="E25" t="n">
-        <v>12.18304729394199</v>
+        <v>12.18319423018658</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>46006</v>
+      </c>
+      <c r="B26" t="n">
+        <v>102259</v>
+      </c>
+      <c r="C26" t="n">
+        <v>318536785</v>
+      </c>
+      <c r="D26" t="n">
+        <v>2964.18310546875</v>
+      </c>
+      <c r="E26" t="n">
+        <v>10.47037706090311</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>46013</v>
+      </c>
+      <c r="B27" t="n">
+        <v>98852</v>
+      </c>
+      <c r="C27" t="n">
+        <v>294578960</v>
+      </c>
+      <c r="D27" t="n">
+        <v>3006.07373046875</v>
+      </c>
+      <c r="E27" t="n">
+        <v>10.29447685177533</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>46020</v>
+      </c>
+      <c r="B28" t="n">
+        <v>44463</v>
+      </c>
+      <c r="C28" t="n">
+        <v>131610480</v>
+      </c>
+      <c r="D28" t="n">
+        <v>2934.538330078125</v>
+      </c>
+      <c r="E28" t="n">
+        <v>6.904161347864301</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>46027</v>
+      </c>
+      <c r="B29" t="n">
+        <v>32977</v>
+      </c>
+      <c r="C29" t="n">
+        <v>100579850</v>
+      </c>
+      <c r="D29" t="n">
+        <v>3226.13037109375</v>
+      </c>
+      <c r="E29" t="n">
+        <v>5.945893461702672</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>46034</v>
+      </c>
+      <c r="B30" t="n">
+        <v>24266</v>
+      </c>
+      <c r="C30" t="n">
+        <v>76923220</v>
+      </c>
+      <c r="D30" t="n">
+        <v>3092.3251953125</v>
+      </c>
+      <c r="E30" t="n">
+        <v>5.100475288451123</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>46041</v>
+      </c>
+      <c r="B31" t="n">
+        <v>35268</v>
+      </c>
+      <c r="C31" t="n">
+        <v>116540860</v>
+      </c>
+      <c r="D31" t="n">
+        <v>3186.62109375</v>
+      </c>
+      <c r="E31" t="n">
+        <v>6.148964237693208</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>46048</v>
+      </c>
+      <c r="B32" t="n">
+        <v>40302</v>
+      </c>
+      <c r="C32" t="n">
+        <v>120099960</v>
+      </c>
+      <c r="D32" t="n">
+        <v>2926.45703125</v>
+      </c>
+      <c r="E32" t="n">
+        <v>6.573169788449224</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>46055</v>
+      </c>
+      <c r="B33" t="n">
+        <v>41788</v>
+      </c>
+      <c r="C33" t="n">
+        <v>141404692</v>
+      </c>
+      <c r="D33" t="n">
+        <v>2344.356689453125</v>
+      </c>
+      <c r="E33" t="n">
+        <v>6.693254584851253</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>46062</v>
+      </c>
+      <c r="B34" t="n">
+        <v>40613</v>
+      </c>
+      <c r="C34" t="n">
+        <v>88536340</v>
+      </c>
+      <c r="D34" t="n">
+        <v>2103.567626953125</v>
+      </c>
+      <c r="E34" t="n">
+        <v>6.598482765481575</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>46070</v>
+      </c>
+      <c r="B35" t="n">
+        <v>45759</v>
+      </c>
+      <c r="C35" t="n">
+        <v>91289205</v>
+      </c>
+      <c r="D35" t="n">
+        <v>1992.1943359375</v>
+      </c>
+      <c r="E35" t="n">
+        <v>7.004059287755366</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>46076</v>
+      </c>
+      <c r="B36" t="n">
+        <v>51162</v>
+      </c>
+      <c r="C36" t="n">
+        <v>97463610</v>
+      </c>
+      <c r="D36" t="n">
+        <v>1855.502807617188</v>
+      </c>
+      <c r="E36" t="n">
+        <v>7.406027286640194</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>46083</v>
+      </c>
+      <c r="B37" t="n">
+        <v>50928</v>
+      </c>
+      <c r="C37" t="n">
+        <v>99920736</v>
+      </c>
+      <c r="D37" t="n">
+        <v>2027.268920898438</v>
+      </c>
+      <c r="E37" t="n">
+        <v>7.389071376979862</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>46090</v>
+      </c>
+      <c r="B38" t="n">
+        <v>60976</v>
+      </c>
+      <c r="C38" t="n">
+        <v>122866640</v>
+      </c>
+      <c r="D38" t="n">
+        <v>1992.938232421875</v>
+      </c>
+      <c r="E38" t="n">
+        <v>8.085204645451292</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>46097</v>
+      </c>
+      <c r="B39" t="n">
+        <v>60999</v>
+      </c>
+      <c r="C39" t="n">
+        <v>128829888</v>
+      </c>
+      <c r="D39" t="n">
+        <v>2351.176025390625</v>
+      </c>
+      <c r="E39" t="n">
+        <v>8.086729361522073</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>46104</v>
+      </c>
+      <c r="B40" t="n">
+        <v>65341</v>
+      </c>
+      <c r="C40" t="n">
+        <v>141201901</v>
+      </c>
+      <c r="D40" t="n">
+        <v>2152.14599609375</v>
+      </c>
+      <c r="E40" t="n">
+        <v>8.369594928536044</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>46111</v>
+      </c>
+      <c r="B41" t="n">
+        <v>71179</v>
+      </c>
+      <c r="C41" t="n">
+        <v>147554067</v>
+      </c>
+      <c r="D41" t="n">
+        <v>2023.514892578125</v>
+      </c>
+      <c r="E41" t="n">
+        <v>8.735494452971144</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B42" t="n">
+        <v>71252</v>
+      </c>
+      <c r="C42" t="n">
+        <v>148210400</v>
+      </c>
+      <c r="D42" t="n">
+        <v>2107.761474609375</v>
+      </c>
+      <c r="E42" t="n">
+        <v>8.739972794037378</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B43" t="n">
+        <v>71524</v>
+      </c>
+      <c r="C43" t="n">
+        <v>158497184</v>
+      </c>
+      <c r="D43" t="n">
+        <v>2370.71484375</v>
+      </c>
+      <c r="E43" t="n">
+        <v>8.756639050059672</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>46132</v>
+      </c>
+      <c r="B44" t="n">
+        <v>101627</v>
+      </c>
+      <c r="C44" t="n">
+        <v>236689283</v>
+      </c>
+      <c r="D44" t="n">
+        <v>2315.21240234375</v>
+      </c>
+      <c r="E44" t="n">
+        <v>10.43797143229205</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B45" t="n">
+        <v>101901</v>
+      </c>
+      <c r="C45" t="n">
+        <v>237531231</v>
+      </c>
+      <c r="D45" t="n">
+        <v>2303.06396484375</v>
+      </c>
+      <c r="E45" t="n">
+        <v>10.45203304499461</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B46" t="n">
+        <v>101745</v>
+      </c>
+      <c r="C46" t="n">
+        <v>238182090</v>
+      </c>
+      <c r="D46" t="n">
+        <v>2346.39697265625</v>
+      </c>
+      <c r="E46" t="n">
+        <v>10.44402948432366</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46153</v>
+      </c>
+      <c r="B47" t="n">
+        <v>26659</v>
+      </c>
+      <c r="C47" t="n">
+        <v>61688926</v>
+      </c>
+      <c r="D47" t="n">
+        <v>2339.36083984375</v>
+      </c>
+      <c r="E47" t="n">
+        <v>5.346055689600105</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B48" t="n">
+        <v>71672</v>
+      </c>
+      <c r="C48" t="n">
+        <v>161477016</v>
+      </c>
+      <c r="D48" t="n">
+        <v>2128.51611328125</v>
+      </c>
+      <c r="E48" t="n">
+        <v>8.765694142398287</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>46168</v>
+      </c>
+      <c r="B49" t="n">
+        <v>111942</v>
+      </c>
+      <c r="C49" t="n">
+        <v>241000000</v>
+      </c>
+      <c r="D49" t="n">
+        <v>2070.858154296875</v>
+      </c>
+      <c r="E49" t="n">
+        <v>10.95489153890127</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B50" t="n">
+        <v>26497</v>
+      </c>
+      <c r="C50" t="n">
+        <v>52270049</v>
+      </c>
+      <c r="D50" t="n">
+        <v>2003.22119140625</v>
+      </c>
+      <c r="E50" t="n">
+        <v>5.329787623599513</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B51" t="n">
+        <v>126971</v>
+      </c>
+      <c r="C51" t="n">
+        <v>209248208</v>
+      </c>
+      <c r="D51" t="n">
+        <v>1690.148559570312</v>
+      </c>
+      <c r="E51" t="n">
+        <v>11.66712420181261</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B52" t="n">
+        <v>76881</v>
+      </c>
+      <c r="C52" t="n">
+        <v>133388535</v>
+      </c>
+      <c r="D52" t="n">
+        <v>1794.961181640625</v>
+      </c>
+      <c r="E52" t="n">
+        <v>9.07864559842187</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B53" t="n">
+        <v>52203</v>
+      </c>
+      <c r="C53" t="n">
+        <v>90989829</v>
+      </c>
+      <c r="D53" t="n">
+        <v>1726.510864257812</v>
+      </c>
+      <c r="E53" t="n">
+        <v>7.480993579416692</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B54" t="n">
+        <v>27084</v>
+      </c>
+      <c r="C54" t="n">
+        <v>46103102</v>
+      </c>
+      <c r="D54" t="n">
+        <v>1610.205810546875</v>
+      </c>
+      <c r="E54" t="n">
+        <v>5.388500825216838</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>46209</v>
+      </c>
+      <c r="B55" t="n">
+        <v>42197</v>
+      </c>
+      <c r="C55" t="n">
+        <v>71903688</v>
+      </c>
+      <c r="D55" t="n">
+        <v>1797.57373046875</v>
+      </c>
+      <c r="E55" t="n">
+        <v>6.725929937659618</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B56" t="n">
+        <v>27801</v>
+      </c>
+      <c r="C56" t="n">
+        <v>48401541</v>
+      </c>
+      <c r="D56" t="n">
+        <v>1773.500732421875</v>
+      </c>
+      <c r="E56" t="n">
+        <v>5.459360334408695</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B57" t="n">
+        <v>7430</v>
+      </c>
+      <c r="C57" t="n">
+        <v>13522600</v>
+      </c>
+      <c r="D57" t="n">
+        <v>1903.758911132812</v>
+      </c>
+      <c r="E57" t="n">
+        <v>2.822318080807614</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B58" t="n">
+        <v>9946</v>
+      </c>
+      <c r="C58" t="n">
+        <v>17853070</v>
+      </c>
+      <c r="D58" t="n">
+        <v>1890.613525390625</v>
+      </c>
+      <c r="E58" t="n">
+        <v>3.265395414805139</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B59" t="n">
+        <v>10399</v>
+      </c>
+      <c r="C59" t="n">
+        <v>19695706</v>
+      </c>
+      <c r="D59" t="n">
+        <v>1858.256469726562</v>
+      </c>
+      <c r="E59" t="n">
+        <v>3.338930199818218</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>46244</v>
+      </c>
+      <c r="B60" t="n">
+        <v>7391</v>
+      </c>
+      <c r="C60" t="n">
+        <v>13998554</v>
+      </c>
+      <c r="D60" t="n">
+        <v>1871.278686523438</v>
+      </c>
+      <c r="E60" t="n">
+        <v>2.814901174676339</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B61" t="n">
+        <v>9926</v>
+      </c>
+      <c r="C61" t="n">
+        <v>7548000</v>
+      </c>
+      <c r="D61" t="n">
+        <v>1912.2021484375</v>
+      </c>
+      <c r="E61" t="n">
+        <v>3.262110638382958</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>46258</v>
+      </c>
+      <c r="B62" t="n">
+        <v>32447</v>
+      </c>
+      <c r="C62" t="n">
+        <v>72778621</v>
+      </c>
+      <c r="D62" t="n">
+        <v>2481.831298828125</v>
+      </c>
+      <c r="E62" t="n">
+        <v>5.897919295096462</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>46265</v>
+      </c>
+      <c r="B63" t="n">
+        <v>53501</v>
+      </c>
+      <c r="C63" t="n">
+        <v>130542440</v>
+      </c>
+      <c r="D63" t="n">
+        <v>2466.8203125</v>
+      </c>
+      <c r="E63" t="n">
+        <v>7.573427999533665</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>46272</v>
+      </c>
+      <c r="B64" t="n">
+        <v>28086</v>
+      </c>
+      <c r="C64" t="n">
+        <v>68923044</v>
+      </c>
+      <c r="D64" t="n">
+        <v>2490.9580078125</v>
+      </c>
+      <c r="E64" t="n">
+        <v>5.48727210753375</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B65" t="n">
+        <v>27180</v>
+      </c>
+      <c r="C65" t="n">
+        <v>66781260</v>
+      </c>
+      <c r="D65" t="n">
+        <v>2514.406982421875</v>
+      </c>
+      <c r="E65" t="n">
+        <v>5.398042224145941</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B66" t="n">
+        <v>27562</v>
+      </c>
+      <c r="C66" t="n">
+        <v>68905000</v>
+      </c>
+      <c r="D66" t="n">
+        <v>2776.46826171875</v>
+      </c>
+      <c r="E66" t="n">
+        <v>5.435843131940453</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B67" t="n">
+        <v>17362</v>
+      </c>
+      <c r="C67" t="n">
+        <v>42000000</v>
+      </c>
+      <c r="D67" t="n">
+        <v>2688.668701171875</v>
+      </c>
+      <c r="E67" t="n">
+        <v>4.314310789187374</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B68" t="n">
+        <v>15112</v>
+      </c>
+      <c r="C68" t="n">
+        <v>40726840</v>
+      </c>
+      <c r="D68" t="n">
+        <v>2711.031494140625</v>
+      </c>
+      <c r="E68" t="n">
+        <v>4.025061529100444</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B69" t="n">
+        <v>12532</v>
+      </c>
+      <c r="C69" t="n">
+        <v>31355064</v>
+      </c>
+      <c r="D69" t="n">
+        <v>2444.357421875</v>
+      </c>
+      <c r="E69" t="n">
+        <v>3.665403112037513</v>
       </c>
     </row>
   </sheetData>

</xml_diff>